<commit_message>
data: hourly update 2026-07-03 10:49Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-07-03.xlsx
+++ b/data/output/workbook/2026-07-03.xlsx
@@ -490,7 +490,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10125075" cy="10344150"/>
+    <ext cx="10125075" cy="10763250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -953,7 +953,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03 04:06</t>
+          <t>2026-07-03 06:49</t>
         </is>
       </c>
     </row>
@@ -2065,7 +2065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q80"/>
+  <dimension ref="A1:Q82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2082,324 +2082,174 @@
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="29" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="29" t="inlineStr">
         <is>
           <t>Chicago White Sox offense vs Cleveland Guardians defense</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="30" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="30" t="inlineStr">
         <is>
           <t>Stat</t>
         </is>
       </c>
-      <c r="B67" s="30" t="inlineStr">
+      <c r="B69" s="30" t="inlineStr">
         <is>
           <t>A Season</t>
         </is>
       </c>
-      <c r="C67" s="30" t="inlineStr">
+      <c r="C69" s="30" t="inlineStr">
         <is>
           <t>A L30</t>
         </is>
       </c>
-      <c r="D67" s="30" t="inlineStr">
+      <c r="D69" s="30" t="inlineStr">
         <is>
           <t>A L20</t>
         </is>
       </c>
-      <c r="E67" s="30" t="inlineStr">
+      <c r="E69" s="30" t="inlineStr">
         <is>
           <t>A L15</t>
         </is>
       </c>
-      <c r="F67" s="30" t="inlineStr">
+      <c r="F69" s="30" t="inlineStr">
         <is>
           <t>A L10</t>
         </is>
       </c>
-      <c r="G67" s="30" t="inlineStr">
+      <c r="G69" s="30" t="inlineStr">
         <is>
           <t>A L5</t>
         </is>
       </c>
-      <c r="H67" s="30" t="inlineStr">
+      <c r="H69" s="30" t="inlineStr">
         <is>
           <t>A Rk</t>
         </is>
       </c>
-      <c r="I67" s="30" t="inlineStr">
+      <c r="I69" s="30" t="inlineStr">
         <is>
           <t>Adv</t>
         </is>
       </c>
-      <c r="J67" s="30" t="inlineStr">
+      <c r="J69" s="30" t="inlineStr">
         <is>
           <t>H Rk</t>
         </is>
       </c>
-      <c r="K67" s="30" t="inlineStr">
+      <c r="K69" s="30" t="inlineStr">
         <is>
           <t>H L5</t>
         </is>
       </c>
-      <c r="L67" s="30" t="inlineStr">
+      <c r="L69" s="30" t="inlineStr">
         <is>
           <t>H L10</t>
         </is>
       </c>
-      <c r="M67" s="30" t="inlineStr">
+      <c r="M69" s="30" t="inlineStr">
         <is>
           <t>H L15</t>
         </is>
       </c>
-      <c r="N67" s="30" t="inlineStr">
+      <c r="N69" s="30" t="inlineStr">
         <is>
           <t>H L20</t>
         </is>
       </c>
-      <c r="O67" s="30" t="inlineStr">
+      <c r="O69" s="30" t="inlineStr">
         <is>
           <t>H L30</t>
         </is>
       </c>
-      <c r="P67" s="30" t="inlineStr">
+      <c r="P69" s="30" t="inlineStr">
         <is>
           <t>H Season</t>
         </is>
       </c>
-      <c r="Q67" s="30" t="inlineStr">
+      <c r="Q69" s="30" t="inlineStr">
         <is>
           <t>Opp stat</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="31" t="inlineStr">
-        <is>
-          <t>Runs/G</t>
-        </is>
-      </c>
-      <c r="B68" s="32" t="n">
-        <v>4.933</v>
-      </c>
-      <c r="C68" s="32" t="n">
-        <v>5.1</v>
-      </c>
-      <c r="D68" s="32" t="n">
-        <v>4.95</v>
-      </c>
-      <c r="E68" s="32" t="n">
-        <v>5.333</v>
-      </c>
-      <c r="F68" s="32" t="n">
-        <v>6.2</v>
-      </c>
-      <c r="G68" s="32" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="H68" s="33" t="inlineStr">
-        <is>
-          <t>11th</t>
-        </is>
-      </c>
-      <c r="I68" s="32" t="inlineStr">
-        <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="J68" s="33" t="inlineStr">
-        <is>
-          <t>16th</t>
-        </is>
-      </c>
-      <c r="K68" s="32" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="L68" s="32" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="M68" s="32" t="n">
-        <v>4.267</v>
-      </c>
-      <c r="N68" s="32" t="n">
-        <v>4</v>
-      </c>
-      <c r="O68" s="32" t="n">
-        <v>4.367</v>
-      </c>
-      <c r="P68" s="32" t="n">
-        <v>4.141</v>
-      </c>
-      <c r="Q68" s="35" t="inlineStr">
-        <is>
-          <t>Opp Runs/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="31" t="inlineStr">
-        <is>
-          <t>Hits/G</t>
-        </is>
-      </c>
-      <c r="B69" s="32" t="n">
-        <v>7.792</v>
-      </c>
-      <c r="C69" s="32" t="n">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="D69" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E69" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F69" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G69" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H69" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I69" s="32" t="inlineStr"/>
-      <c r="J69" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K69" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L69" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M69" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N69" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O69" s="32" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="P69" s="32" t="n">
-        <v>7.939</v>
-      </c>
-      <c r="Q69" s="35" t="inlineStr">
-        <is>
-          <t>Opp Hits/G</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="31" t="inlineStr">
         <is>
-          <t>HR/G</t>
+          <t>Runs/G</t>
         </is>
       </c>
       <c r="B70" s="32" t="n">
-        <v>1.354</v>
+        <v>4.933</v>
       </c>
       <c r="C70" s="32" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="D70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H70" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I70" s="32" t="inlineStr"/>
-      <c r="J70" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>5.1</v>
+      </c>
+      <c r="D70" s="32" t="n">
+        <v>4.95</v>
+      </c>
+      <c r="E70" s="32" t="n">
+        <v>5.333</v>
+      </c>
+      <c r="F70" s="32" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="G70" s="32" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="H70" s="33" t="inlineStr">
+        <is>
+          <t>11th</t>
+        </is>
+      </c>
+      <c r="I70" s="32" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="J70" s="33" t="inlineStr">
+        <is>
+          <t>16th</t>
+        </is>
+      </c>
+      <c r="K70" s="32" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="L70" s="32" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="M70" s="32" t="n">
+        <v>4.267</v>
+      </c>
+      <c r="N70" s="32" t="n">
+        <v>4</v>
       </c>
       <c r="O70" s="32" t="n">
-        <v>0.75</v>
+        <v>4.367</v>
       </c>
       <c r="P70" s="32" t="n">
-        <v>1.143</v>
+        <v>4.141</v>
       </c>
       <c r="Q70" s="35" t="inlineStr">
         <is>
-          <t>Opp HR/G</t>
+          <t>Opp Runs/G</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="31" t="inlineStr">
         <is>
-          <t>Batter K/G</t>
+          <t>Hits/G</t>
         </is>
       </c>
       <c r="B71" s="32" t="n">
-        <v>9.208</v>
+        <v>7.792</v>
       </c>
       <c r="C71" s="32" t="n">
-        <v>7.8</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="D71" s="32" t="inlineStr">
         <is>
@@ -2453,390 +2303,390 @@
         </is>
       </c>
       <c r="O71" s="32" t="n">
-        <v>9.5</v>
+        <v>10.5</v>
       </c>
       <c r="P71" s="32" t="n">
-        <v>9.388</v>
+        <v>7.939</v>
       </c>
       <c r="Q71" s="35" t="inlineStr">
         <is>
-          <t>Opp Batter K/G</t>
+          <t>Opp Hits/G</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="31" t="inlineStr">
         <is>
+          <t>HR/G</t>
+        </is>
+      </c>
+      <c r="B72" s="32" t="n">
+        <v>1.354</v>
+      </c>
+      <c r="C72" s="32" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="D72" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E72" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F72" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G72" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H72" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I72" s="32" t="inlineStr"/>
+      <c r="J72" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K72" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L72" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M72" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N72" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O72" s="32" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="P72" s="32" t="n">
+        <v>1.143</v>
+      </c>
+      <c r="Q72" s="35" t="inlineStr">
+        <is>
+          <t>Opp HR/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="31" t="inlineStr">
+        <is>
+          <t>Batter K/G</t>
+        </is>
+      </c>
+      <c r="B73" s="32" t="n">
+        <v>9.208</v>
+      </c>
+      <c r="C73" s="32" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="D73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H73" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I73" s="32" t="inlineStr"/>
+      <c r="J73" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O73" s="32" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="P73" s="32" t="n">
+        <v>9.388</v>
+      </c>
+      <c r="Q73" s="35" t="inlineStr">
+        <is>
+          <t>Opp Batter K/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="31" t="inlineStr">
+        <is>
           <t>1st Inn R/G</t>
         </is>
       </c>
-      <c r="B72" s="32" t="n">
+      <c r="B74" s="32" t="n">
         <v>0.589</v>
       </c>
-      <c r="C72" s="32" t="n">
+      <c r="C74" s="32" t="n">
         <v>0.6</v>
       </c>
-      <c r="D72" s="32" t="n">
+      <c r="D74" s="32" t="n">
         <v>0.4</v>
       </c>
-      <c r="E72" s="32" t="n">
+      <c r="E74" s="32" t="n">
         <v>0.4</v>
       </c>
-      <c r="F72" s="32" t="n">
+      <c r="F74" s="32" t="n">
         <v>0.4</v>
       </c>
-      <c r="G72" s="32" t="n">
+      <c r="G74" s="32" t="n">
         <v>0.8</v>
       </c>
-      <c r="H72" s="34" t="inlineStr">
+      <c r="H74" s="34" t="inlineStr">
         <is>
           <t>7th</t>
         </is>
       </c>
-      <c r="I72" s="32" t="inlineStr"/>
-      <c r="J72" s="34" t="inlineStr">
+      <c r="I74" s="32" t="inlineStr"/>
+      <c r="J74" s="34" t="inlineStr">
         <is>
           <t>3rd</t>
         </is>
       </c>
-      <c r="K72" s="32" t="n">
+      <c r="K74" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="L72" s="32" t="n">
+      <c r="L74" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="M72" s="32" t="n">
+      <c r="M74" s="32" t="n">
         <v>0.333</v>
       </c>
-      <c r="N72" s="32" t="n">
+      <c r="N74" s="32" t="n">
         <v>0.3</v>
       </c>
-      <c r="O72" s="32" t="n">
+      <c r="O74" s="32" t="n">
         <v>0.367</v>
       </c>
-      <c r="P72" s="32" t="n">
+      <c r="P74" s="32" t="n">
         <v>0.36</v>
       </c>
-      <c r="Q72" s="35" t="inlineStr">
+      <c r="Q74" s="35" t="inlineStr">
         <is>
           <t>Opp 1st Inn R/G</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="29" t="inlineStr">
+    <row r="76">
+      <c r="A76" s="29" t="inlineStr">
         <is>
           <t>Cleveland Guardians offense vs Chicago White Sox defense</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="30" t="inlineStr">
+    <row r="77">
+      <c r="A77" s="30" t="inlineStr">
         <is>
           <t>Stat</t>
         </is>
       </c>
-      <c r="B75" s="30" t="inlineStr">
+      <c r="B77" s="30" t="inlineStr">
         <is>
           <t>A Season</t>
         </is>
       </c>
-      <c r="C75" s="30" t="inlineStr">
+      <c r="C77" s="30" t="inlineStr">
         <is>
           <t>A L30</t>
         </is>
       </c>
-      <c r="D75" s="30" t="inlineStr">
+      <c r="D77" s="30" t="inlineStr">
         <is>
           <t>A L20</t>
         </is>
       </c>
-      <c r="E75" s="30" t="inlineStr">
+      <c r="E77" s="30" t="inlineStr">
         <is>
           <t>A L15</t>
         </is>
       </c>
-      <c r="F75" s="30" t="inlineStr">
+      <c r="F77" s="30" t="inlineStr">
         <is>
           <t>A L10</t>
         </is>
       </c>
-      <c r="G75" s="30" t="inlineStr">
+      <c r="G77" s="30" t="inlineStr">
         <is>
           <t>A L5</t>
         </is>
       </c>
-      <c r="H75" s="30" t="inlineStr">
+      <c r="H77" s="30" t="inlineStr">
         <is>
           <t>A Rk</t>
         </is>
       </c>
-      <c r="I75" s="30" t="inlineStr">
+      <c r="I77" s="30" t="inlineStr">
         <is>
           <t>Adv</t>
         </is>
       </c>
-      <c r="J75" s="30" t="inlineStr">
+      <c r="J77" s="30" t="inlineStr">
         <is>
           <t>H Rk</t>
         </is>
       </c>
-      <c r="K75" s="30" t="inlineStr">
+      <c r="K77" s="30" t="inlineStr">
         <is>
           <t>H L5</t>
         </is>
       </c>
-      <c r="L75" s="30" t="inlineStr">
+      <c r="L77" s="30" t="inlineStr">
         <is>
           <t>H L10</t>
         </is>
       </c>
-      <c r="M75" s="30" t="inlineStr">
+      <c r="M77" s="30" t="inlineStr">
         <is>
           <t>H L15</t>
         </is>
       </c>
-      <c r="N75" s="30" t="inlineStr">
+      <c r="N77" s="30" t="inlineStr">
         <is>
           <t>H L20</t>
         </is>
       </c>
-      <c r="O75" s="30" t="inlineStr">
+      <c r="O77" s="30" t="inlineStr">
         <is>
           <t>H L30</t>
         </is>
       </c>
-      <c r="P75" s="30" t="inlineStr">
+      <c r="P77" s="30" t="inlineStr">
         <is>
           <t>H Season</t>
         </is>
       </c>
-      <c r="Q75" s="30" t="inlineStr">
+      <c r="Q77" s="30" t="inlineStr">
         <is>
           <t>Opp stat</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="31" t="inlineStr">
-        <is>
-          <t>Runs/G</t>
-        </is>
-      </c>
-      <c r="B76" s="32" t="n">
-        <v>3.949</v>
-      </c>
-      <c r="C76" s="32" t="n">
-        <v>3.7</v>
-      </c>
-      <c r="D76" s="32" t="n">
-        <v>3.7</v>
-      </c>
-      <c r="E76" s="32" t="n">
-        <v>4.067</v>
-      </c>
-      <c r="F76" s="32" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="G76" s="32" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="H76" s="33" t="inlineStr">
-        <is>
-          <t>13th</t>
-        </is>
-      </c>
-      <c r="I76" s="32" t="inlineStr"/>
-      <c r="J76" s="33" t="inlineStr">
-        <is>
-          <t>14th</t>
-        </is>
-      </c>
-      <c r="K76" s="32" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="L76" s="32" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="M76" s="32" t="n">
-        <v>3.867</v>
-      </c>
-      <c r="N76" s="32" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="O76" s="32" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="P76" s="32" t="n">
-        <v>4.733</v>
-      </c>
-      <c r="Q76" s="35" t="inlineStr">
-        <is>
-          <t>Opp Runs/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="31" t="inlineStr">
-        <is>
-          <t>Hits/G</t>
-        </is>
-      </c>
-      <c r="B77" s="32" t="n">
-        <v>7.735</v>
-      </c>
-      <c r="C77" s="32" t="n">
-        <v>9.75</v>
-      </c>
-      <c r="D77" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E77" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F77" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G77" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H77" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I77" s="32" t="inlineStr"/>
-      <c r="J77" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K77" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L77" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M77" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N77" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O77" s="32" t="n">
-        <v>7</v>
-      </c>
-      <c r="P77" s="32" t="n">
-        <v>7.854</v>
-      </c>
-      <c r="Q77" s="35" t="inlineStr">
-        <is>
-          <t>Opp Hits/G</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="31" t="inlineStr">
         <is>
-          <t>HR/G</t>
+          <t>Runs/G</t>
         </is>
       </c>
       <c r="B78" s="32" t="n">
-        <v>0.959</v>
+        <v>3.949</v>
       </c>
       <c r="C78" s="32" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="D78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H78" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
+        <v>3.7</v>
+      </c>
+      <c r="D78" s="32" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="E78" s="32" t="n">
+        <v>4.067</v>
+      </c>
+      <c r="F78" s="32" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="G78" s="32" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="H78" s="33" t="inlineStr">
+        <is>
+          <t>13th</t>
         </is>
       </c>
       <c r="I78" s="32" t="inlineStr"/>
-      <c r="J78" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J78" s="33" t="inlineStr">
+        <is>
+          <t>14th</t>
+        </is>
+      </c>
+      <c r="K78" s="32" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="L78" s="32" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="M78" s="32" t="n">
+        <v>3.867</v>
+      </c>
+      <c r="N78" s="32" t="n">
+        <v>4.2</v>
       </c>
       <c r="O78" s="32" t="n">
-        <v>0.6</v>
+        <v>4.3</v>
       </c>
       <c r="P78" s="32" t="n">
-        <v>1.062</v>
+        <v>4.733</v>
       </c>
       <c r="Q78" s="35" t="inlineStr">
         <is>
-          <t>Opp HR/G</t>
+          <t>Opp Runs/G</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="31" t="inlineStr">
         <is>
-          <t>Batter K/G</t>
+          <t>Hits/G</t>
         </is>
       </c>
       <c r="B79" s="32" t="n">
-        <v>8</v>
+        <v>7.735</v>
       </c>
       <c r="C79" s="32" t="n">
-        <v>11.25</v>
+        <v>9.75</v>
       </c>
       <c r="D79" s="32" t="inlineStr">
         <is>
@@ -2890,71 +2740,221 @@
         </is>
       </c>
       <c r="O79" s="32" t="n">
-        <v>7.2</v>
+        <v>7</v>
       </c>
       <c r="P79" s="32" t="n">
-        <v>7.938</v>
+        <v>7.854</v>
       </c>
       <c r="Q79" s="35" t="inlineStr">
         <is>
-          <t>Opp Batter K/G</t>
+          <t>Opp Hits/G</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="31" t="inlineStr">
         <is>
+          <t>HR/G</t>
+        </is>
+      </c>
+      <c r="B80" s="32" t="n">
+        <v>0.959</v>
+      </c>
+      <c r="C80" s="32" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D80" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E80" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F80" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G80" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H80" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I80" s="32" t="inlineStr"/>
+      <c r="J80" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K80" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L80" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M80" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N80" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O80" s="32" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="P80" s="32" t="n">
+        <v>1.062</v>
+      </c>
+      <c r="Q80" s="35" t="inlineStr">
+        <is>
+          <t>Opp HR/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="31" t="inlineStr">
+        <is>
+          <t>Batter K/G</t>
+        </is>
+      </c>
+      <c r="B81" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C81" s="32" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="D81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H81" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I81" s="32" t="inlineStr"/>
+      <c r="J81" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O81" s="32" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="P81" s="32" t="n">
+        <v>7.938</v>
+      </c>
+      <c r="Q81" s="35" t="inlineStr">
+        <is>
+          <t>Opp Batter K/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="31" t="inlineStr">
+        <is>
           <t>1st Inn R/G</t>
         </is>
       </c>
-      <c r="B80" s="32" t="n">
+      <c r="B82" s="32" t="n">
         <v>0.507</v>
       </c>
-      <c r="C80" s="32" t="n">
+      <c r="C82" s="32" t="n">
         <v>0.367</v>
       </c>
-      <c r="D80" s="32" t="n">
+      <c r="D82" s="32" t="n">
         <v>0.25</v>
       </c>
-      <c r="E80" s="32" t="n">
+      <c r="E82" s="32" t="n">
         <v>0.267</v>
       </c>
-      <c r="F80" s="32" t="n">
+      <c r="F82" s="32" t="n">
         <v>0.3</v>
       </c>
-      <c r="G80" s="32" t="n">
+      <c r="G82" s="32" t="n">
         <v>0.4</v>
       </c>
-      <c r="H80" s="33" t="inlineStr">
+      <c r="H82" s="33" t="inlineStr">
         <is>
           <t>18th</t>
         </is>
       </c>
-      <c r="I80" s="32" t="inlineStr"/>
-      <c r="J80" s="33" t="inlineStr">
+      <c r="I82" s="32" t="inlineStr"/>
+      <c r="J82" s="33" t="inlineStr">
         <is>
           <t>18th</t>
         </is>
       </c>
-      <c r="K80" s="32" t="n">
+      <c r="K82" s="32" t="n">
         <v>0.6</v>
       </c>
-      <c r="L80" s="32" t="n">
+      <c r="L82" s="32" t="n">
         <v>0.3</v>
       </c>
-      <c r="M80" s="32" t="n">
+      <c r="M82" s="32" t="n">
         <v>0.467</v>
       </c>
-      <c r="N80" s="32" t="n">
+      <c r="N82" s="32" t="n">
         <v>0.55</v>
       </c>
-      <c r="O80" s="32" t="n">
+      <c r="O82" s="32" t="n">
         <v>0.533</v>
       </c>
-      <c r="P80" s="32" t="n">
+      <c r="P82" s="32" t="n">
         <v>0.548</v>
       </c>
-      <c r="Q80" s="35" t="inlineStr">
+      <c r="Q82" s="35" t="inlineStr">
         <is>
           <t>Opp 1st Inn R/G</t>
         </is>
@@ -7747,13 +7747,13 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.6952962962962962</v>
+        <v>0.6928897338403042</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-228</v>
+        <v>-226</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -7777,7 +7777,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 69.5% (fair -228). Your call.</t>
+          <t>Model 69.3% (fair -226). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -7879,10 +7879,10 @@
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.6199629629629629</v>
+        <v>0.6174444444444445</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-163</v>
+        <v>-161</v>
       </c>
       <c r="H7" s="15" t="n">
         <v>170</v>
@@ -7909,7 +7909,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 62.0% (fair -163). Your call.</t>
+          <t>Model 61.7% (fair -161). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -8058,12 +8058,12 @@
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>Minnesota Twins @ New York Yankees</t>
+          <t>Pittsburgh Pirates @ Washington Nationals</t>
         </is>
       </c>
       <c r="C10" s="20" t="inlineStr">
         <is>
-          <t>23:05</t>
+          <t>22:45</t>
         </is>
       </c>
       <c r="D10" s="20" t="inlineStr">
@@ -8073,17 +8073,17 @@
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>Minnesota Twins +1.5</t>
+          <t>Pittsburgh Pirates +1.5</t>
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.59</v>
+        <v>0.6663156398104265</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-144</v>
+        <v>-200</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>128</v>
+        <v>-111</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -8107,7 +8107,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 59.0% (fair -144). Your call.</t>
+          <t>Model 66.6% (fair -200). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -8124,12 +8124,12 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates @ Washington Nationals</t>
+          <t>Boston Red Sox @ Los Angeles Angels</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>22:45</t>
+          <t>01:38</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
@@ -8139,17 +8139,17 @@
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates +1.5</t>
+          <t>Los Angeles Angels -1.5</t>
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.6662943396226416</v>
+        <v>0.4010958904109589</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>-200</v>
+        <v>149</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>-112</v>
+        <v>192</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -8173,7 +8173,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 66.6% (fair -200). Your call.</t>
+          <t>Model 40.1% (fair +149). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -8209,13 +8209,13 @@
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.5353153153153154</v>
+        <v>0.5352995391705069</v>
       </c>
       <c r="G12" s="14" t="n">
         <v>-115</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="I12" s="13">
         <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
@@ -8251,37 +8251,37 @@
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>Boston Red Sox @ Los Angeles Angels</t>
+          <t>Baltimore Orioles @ Cincinnati Reds</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>01:38</t>
+          <t>23:10</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Los Angeles Angels -1.5</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.4010958904109589</v>
+        <v>0.485793991416309</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>149</v>
+        <v>106</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>192</v>
+        <v>133</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -8305,7 +8305,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 40.1% (fair +149). Your call.</t>
+          <t>Model 48.6% (fair +106). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -8317,37 +8317,37 @@
     <row r="14">
       <c r="A14" s="20" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B14" s="20" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates @ Washington Nationals</t>
+          <t>Miami Marlins @ Athletics</t>
         </is>
       </c>
       <c r="C14" s="20" t="inlineStr">
         <is>
-          <t>15:05</t>
+          <t>01:40</t>
         </is>
       </c>
       <c r="D14" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>Athletics -1.5</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.5913622119815668</v>
+        <v>0.4242585551330798</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>-145</v>
+        <v>136</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>-117</v>
+        <v>163</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -8371,7 +8371,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 59.1% (fair -145). Your call.</t>
+          <t>Model 42.4% (fair +136). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -8388,12 +8388,12 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates @ Washington Nationals</t>
+          <t>Minnesota Twins @ New York Yankees</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>22:45</t>
+          <t>23:05</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
@@ -8403,17 +8403,17 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.475304347826087</v>
+        <v>0.3972661870503597</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>110</v>
+        <v>152</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>130</v>
+        <v>178</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -8437,7 +8437,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 47.5% (fair +110). Your call.</t>
+          <t>Model 39.7% (fair +152). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -8454,12 +8454,12 @@
       </c>
       <c r="B16" s="20" t="inlineStr">
         <is>
-          <t>Minnesota Twins @ New York Yankees</t>
+          <t>Pittsburgh Pirates @ Washington Nationals</t>
         </is>
       </c>
       <c r="C16" s="20" t="inlineStr">
         <is>
-          <t>23:05</t>
+          <t>22:45</t>
         </is>
       </c>
       <c r="D16" s="20" t="inlineStr">
@@ -8469,17 +8469,17 @@
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.4005514705882353</v>
+        <v>0.4732618025751073</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>150</v>
+        <v>111</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>172</v>
+        <v>133</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -8503,7 +8503,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 40.1% (fair +150). Your call.</t>
+          <t>Model 47.3% (fair +111). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -8530,22 +8530,22 @@
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>Athletics -1.5</t>
+          <t>Under 10.5</t>
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.4242578125</v>
+        <v>0.5310294117647059</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>136</v>
+        <v>-113</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>156</v>
+        <v>104</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -8569,7 +8569,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 42.4% (fair +136). Your call.</t>
+          <t>Model 53.1% (fair -113). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -8581,37 +8581,37 @@
     <row r="18">
       <c r="A18" s="20" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B18" s="20" t="inlineStr">
         <is>
-          <t>St. Louis Cardinals @ Chicago Cubs</t>
+          <t>Pittsburgh Pirates @ Washington Nationals</t>
         </is>
       </c>
       <c r="C18" s="20" t="inlineStr">
         <is>
-          <t>20:05</t>
+          <t>15:05</t>
         </is>
       </c>
       <c r="D18" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E18" s="20" t="inlineStr">
         <is>
-          <t>Chicago Cubs -1.5</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.423984375</v>
+        <v>0.5944477477477478</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>136</v>
+        <v>-147</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>156</v>
+        <v>-122</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -8635,7 +8635,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 42.4% (fair +136). Your call.</t>
+          <t>Model 59.4% (fair -147). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -8652,32 +8652,32 @@
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>Miami Marlins @ Athletics</t>
+          <t>Baltimore Orioles @ Cincinnati Reds</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>01:40</t>
+          <t>23:10</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Under 10.5</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.5310294117647059</v>
+        <v>0.5724272300469483</v>
       </c>
       <c r="G19" s="14" t="n">
+        <v>-134</v>
+      </c>
+      <c r="H19" s="15" t="n">
         <v>-113</v>
-      </c>
-      <c r="H19" s="15" t="n">
-        <v>104</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -8701,7 +8701,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 53.1% (fair -113). Your call.</t>
+          <t>Model 57.2% (fair -134). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -8713,17 +8713,17 @@
     <row r="20">
       <c r="A20" s="20" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B20" s="20" t="inlineStr">
         <is>
-          <t>Baltimore Orioles @ Cincinnati Reds</t>
+          <t>New York Mets @ Atlanta Braves</t>
         </is>
       </c>
       <c r="C20" s="20" t="inlineStr">
         <is>
-          <t>23:10</t>
+          <t>00:08</t>
         </is>
       </c>
       <c r="D20" s="20" t="inlineStr">
@@ -8733,17 +8733,17 @@
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.5739657276995306</v>
+        <v>0.4073003802281369</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>-135</v>
+        <v>146</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>-113</v>
+        <v>163</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -8767,7 +8767,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 57.4% (fair -135). Your call.</t>
+          <t>Model 40.7% (fair +146). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -8803,10 +8803,10 @@
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.421015625</v>
+        <v>0.4183984374999999</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H21" s="15" t="n">
         <v>156</v>
@@ -8833,7 +8833,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 42.1% (fair +138). Your call.</t>
+          <t>Model 41.8% (fair +139). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -8845,37 +8845,37 @@
     <row r="22">
       <c r="A22" s="20" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B22" s="20" t="inlineStr">
         <is>
-          <t>New York Mets @ Atlanta Braves</t>
+          <t>St. Louis Cardinals @ Chicago Cubs</t>
         </is>
       </c>
       <c r="C22" s="20" t="inlineStr">
         <is>
-          <t>00:08</t>
+          <t>20:05</t>
         </is>
       </c>
       <c r="D22" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E22" s="20" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Under 10.5</t>
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.4079087452471483</v>
+        <v>0.53225</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>145</v>
+        <v>-114</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>163</v>
+        <v>100</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -8899,7 +8899,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 40.8% (fair +145). Your call.</t>
+          <t>Model 53.2% (fair -114). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -8916,32 +8916,32 @@
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>San Francisco Giants @ Colorado Rockies</t>
+          <t>St. Louis Cardinals @ Chicago Cubs</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>00:10</t>
+          <t>20:05</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Chicago Cubs -1.5</t>
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.4358606557377049</v>
+        <v>0.42496</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -8965,7 +8965,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 43.6% (fair +129). Your call.</t>
+          <t>Model 42.5% (fair +135). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -8982,32 +8982,32 @@
       </c>
       <c r="B24" s="20" t="inlineStr">
         <is>
-          <t>St. Louis Cardinals @ Chicago Cubs</t>
+          <t>New York Mets @ Atlanta Braves</t>
         </is>
       </c>
       <c r="C24" s="20" t="inlineStr">
         <is>
-          <t>20:05</t>
+          <t>23:15</t>
         </is>
       </c>
       <c r="D24" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E24" s="20" t="inlineStr">
         <is>
-          <t>Under 10.5</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.5345910891089108</v>
+        <v>0.509326923076923</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>-115</v>
+        <v>-104</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>-102</v>
+        <v>108</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -9031,7 +9031,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 53.5% (fair -115). Your call.</t>
+          <t>Model 50.9% (fair -104). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -9048,32 +9048,32 @@
       </c>
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>New York Mets @ Atlanta Braves</t>
+          <t>Tampa Bay Rays @ Houston Astros</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>23:15</t>
+          <t>00:15</t>
         </is>
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Over 8.5</t>
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.5086538461538461</v>
+        <v>0.5117156862745098</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>-104</v>
+        <v>-105</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -9097,7 +9097,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 50.9% (fair -104). Your call.</t>
+          <t>Model 51.2% (fair -105). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -9133,13 +9133,13 @@
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.5508352112676056</v>
+        <v>0.5501207547169812</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>-123</v>
+        <v>-122</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>-113</v>
+        <v>-112</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -9163,7 +9163,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 55.1% (fair -123). Your call.</t>
+          <t>Model 55.0% (fair -122). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -9180,32 +9180,32 @@
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays @ Houston Astros</t>
+          <t>San Francisco Giants @ Colorado Rockies</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>00:15</t>
+          <t>00:10</t>
         </is>
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>Over 8.5</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.5085784313725491</v>
+        <v>0.4370168067226891</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>-103</v>
+        <v>129</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>104</v>
+        <v>138</v>
       </c>
       <c r="I27" s="13">
         <f>IF($H$27="","",IF($H$27&lt;0,-$H$27/(-$H$27+100),100/($H$27+100)))</f>
@@ -9229,7 +9229,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 50.9% (fair -103). Your call.</t>
+          <t>Model 43.7% (fair +129). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -9246,32 +9246,32 @@
       </c>
       <c r="B28" s="20" t="inlineStr">
         <is>
-          <t>St. Louis Cardinals @ Chicago Cubs</t>
+          <t>Pittsburgh Pirates @ Washington Nationals</t>
         </is>
       </c>
       <c r="C28" s="20" t="inlineStr">
         <is>
-          <t>20:05</t>
+          <t>22:45</t>
         </is>
       </c>
       <c r="D28" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E28" s="20" t="inlineStr">
         <is>
-          <t>St. Louis Cardinals +1.5</t>
+          <t>Over 9.5</t>
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.5759761061946903</v>
+        <v>0.5300941176470588</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-136</v>
+        <v>-113</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>-126</v>
+        <v>-104</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
@@ -9295,7 +9295,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 57.6% (fair -136). Your call.</t>
+          <t>Model 53.0% (fair -113). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -9312,32 +9312,32 @@
       </c>
       <c r="B29" s="12" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays @ Houston Astros</t>
+          <t>Minnesota Twins @ New York Yankees</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
-          <t>00:15</t>
+          <t>23:05</t>
         </is>
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>Minnesota Twins +1.5</t>
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.5065517241379309</v>
+        <v>0.5519943925233645</v>
       </c>
       <c r="G29" s="14" t="n">
-        <v>-103</v>
+        <v>-123</v>
       </c>
       <c r="H29" s="15" t="n">
-        <v>103</v>
+        <v>-114</v>
       </c>
       <c r="I29" s="13">
         <f>IF($H$29="","",IF($H$29&lt;0,-$H$29/(-$H$29+100),100/($H$29+100)))</f>
@@ -9361,7 +9361,7 @@
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>Model 50.7% (fair -103). Your call.</t>
+          <t>Model 55.2% (fair -123). Your call.</t>
         </is>
       </c>
       <c r="O29" s="15" t="n"/>
@@ -9538,13 +9538,13 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.4561111111111111</v>
+        <v>0.4550691244239632</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -9568,7 +9568,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 45.6% (fair +119). Your call.</t>
+          <t>Model 45.5% (fair +120). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -9604,10 +9604,10 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5439152073732718</v>
+        <v>0.5449396313364054</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-119</v>
+        <v>-120</v>
       </c>
       <c r="H6" s="15" t="n">
         <v>-117</v>
@@ -9634,7 +9634,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 54.4% (fair -119). Your call.</t>
+          <t>Model 54.5% (fair -120). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -9670,10 +9670,10 @@
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.46545</v>
+        <v>0.46775</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H7" s="15" t="n">
         <v>100</v>
@@ -9700,7 +9700,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 46.5% (fair +115). Your call.</t>
+          <t>Model 46.8% (fair +114). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -9736,13 +9736,13 @@
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.5345910891089108</v>
+        <v>0.53225</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>-115</v>
+        <v>-114</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>-102</v>
+        <v>100</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -9766,7 +9766,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 53.5% (fair -115). Your call.</t>
+          <t>Model 53.2% (fair -114). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -9802,13 +9802,13 @@
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.423984375</v>
+        <v>0.42496</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -9832,7 +9832,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 42.4% (fair +136). Your call.</t>
+          <t>Model 42.5% (fair +135). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -9868,13 +9868,13 @@
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.5759761061946903</v>
+        <v>0.5750246696035243</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-136</v>
+        <v>-135</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>-126</v>
+        <v>-127</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -9898,7 +9898,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 57.6% (fair -136). Your call.</t>
+          <t>Model 57.5% (fair -135). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -9934,13 +9934,13 @@
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.475304347826087</v>
+        <v>0.4732618025751073</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -9964,7 +9964,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 47.5% (fair +110). Your call.</t>
+          <t>Model 47.3% (fair +111). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -10000,10 +10000,10 @@
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.5246935622317597</v>
+        <v>0.5267484978540773</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>-110</v>
+        <v>-111</v>
       </c>
       <c r="H12" s="15" t="n">
         <v>-133</v>
@@ -10030,7 +10030,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 52.5% (fair -110). Your call.</t>
+          <t>Model 52.7% (fair -111). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -10066,10 +10066,10 @@
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.5769</v>
+        <v>0.5300941176470588</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-136</v>
+        <v>-113</v>
       </c>
       <c r="H13" s="15" t="n">
         <v>-104</v>
@@ -10096,7 +10096,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 57.7% (fair -136). Your call.</t>
+          <t>Model 53.0% (fair -113). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -10132,13 +10132,13 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.4231</v>
+        <v>0.46995</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>136</v>
+        <v>113</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>125</v>
+        <v>100</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -10162,7 +10162,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 42.3% (fair +136). Your call.</t>
+          <t>Model 47.0% (fair +113). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -10264,13 +10264,13 @@
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.6662943396226416</v>
+        <v>0.6663156398104265</v>
       </c>
       <c r="G16" s="14" t="n">
         <v>-200</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>-112</v>
+        <v>-111</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -10330,13 +10330,13 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.4005514705882353</v>
+        <v>0.3972661870503597</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -10360,7 +10360,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 40.1% (fair +150). Your call.</t>
+          <t>Model 39.7% (fair +152). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -10396,10 +10396,10 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.5994744525547445</v>
+        <v>0.6027131386861314</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>-150</v>
+        <v>-152</v>
       </c>
       <c r="H18" s="15" t="n">
         <v>-174</v>
@@ -10426,7 +10426,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 59.9% (fair -150). Your call.</t>
+          <t>Model 60.3% (fair -152). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -10468,7 +10468,7 @@
         <v>121</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>105</v>
+        <v>-102</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -10534,7 +10534,7 @@
         <v>-121</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -10594,10 +10594,10 @@
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.41</v>
+        <v>0.447981220657277</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>144</v>
+        <v>123</v>
       </c>
       <c r="H21" s="15" t="n">
         <v>113</v>
@@ -10624,7 +10624,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 41.0% (fair +144). Your call.</t>
+          <t>Model 44.8% (fair +123). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -10660,13 +10660,13 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.59</v>
+        <v>0.5519943925233645</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-144</v>
+        <v>-123</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>128</v>
+        <v>-114</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -10690,7 +10690,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 59.0% (fair -144). Your call.</t>
+          <t>Model 55.2% (fair -123). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -10726,10 +10726,10 @@
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.5739657276995306</v>
+        <v>0.5724272300469483</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>-135</v>
+        <v>-134</v>
       </c>
       <c r="H23" s="15" t="n">
         <v>-113</v>
@@ -10756,7 +10756,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 57.4% (fair -135). Your call.</t>
+          <t>Model 57.2% (fair -134). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -10792,13 +10792,13 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.426056338028169</v>
+        <v>0.4275829383886255</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -10822,7 +10822,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 42.6% (fair +135). Your call.</t>
+          <t>Model 42.8% (fair +134). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -10864,7 +10864,7 @@
         <v>-113</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -10990,13 +10990,13 @@
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.4582511210762332</v>
+        <v>0.4543859649122807</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="I27" s="13">
         <f>IF($H$27="","",IF($H$27&lt;0,-$H$27/(-$H$27+100),100/($H$27+100)))</f>
@@ -11020,7 +11020,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 45.8% (fair +118). Your call.</t>
+          <t>Model 45.4% (fair +120). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -11056,10 +11056,10 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.5417361233480177</v>
+        <v>0.5456524229074891</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-118</v>
+        <v>-120</v>
       </c>
       <c r="H28" s="15" t="n">
         <v>-127</v>
@@ -11086,7 +11086,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 54.2% (fair -118). Your call.</t>
+          <t>Model 54.6% (fair -120). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -11122,7 +11122,7 @@
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.5347</v>
+        <v>0.5354</v>
       </c>
       <c r="G29" s="14" t="n">
         <v>-115</v>
@@ -11188,7 +11188,7 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.4653</v>
+        <v>0.4646</v>
       </c>
       <c r="G30" s="14" t="n">
         <v>115</v>
@@ -11254,10 +11254,10 @@
         </is>
       </c>
       <c r="F31" s="13" t="n">
-        <v>0.3800380228136883</v>
+        <v>0.3825475285171103</v>
       </c>
       <c r="G31" s="14" t="n">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="H31" s="15" t="n">
         <v>163</v>
@@ -11284,7 +11284,7 @@
       </c>
       <c r="N31" s="19" t="inlineStr">
         <is>
-          <t>Model 38.0% (fair +163). Your call.</t>
+          <t>Model 38.3% (fair +161). Your call.</t>
         </is>
       </c>
       <c r="O31" s="15" t="n"/>
@@ -11320,10 +11320,10 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.6199629629629629</v>
+        <v>0.6174444444444445</v>
       </c>
       <c r="G32" s="14" t="n">
-        <v>-163</v>
+        <v>-161</v>
       </c>
       <c r="H32" s="15" t="n">
         <v>170</v>
@@ -11350,7 +11350,7 @@
       </c>
       <c r="N32" s="19" t="inlineStr">
         <is>
-          <t>Model 62.0% (fair -163). Your call.</t>
+          <t>Model 61.7% (fair -161). Your call.</t>
         </is>
       </c>
       <c r="O32" s="15" t="n"/>
@@ -11386,7 +11386,7 @@
         </is>
       </c>
       <c r="F33" s="13" t="n">
-        <v>0.5086538461538461</v>
+        <v>0.509326923076923</v>
       </c>
       <c r="G33" s="14" t="n">
         <v>-104</v>
@@ -11452,7 +11452,7 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.4913480769230769</v>
+        <v>0.4906730769230769</v>
       </c>
       <c r="G34" s="14" t="n">
         <v>104</v>
@@ -11518,13 +11518,13 @@
         </is>
       </c>
       <c r="F35" s="13" t="n">
-        <v>0.3603</v>
+        <v>0.4016</v>
       </c>
       <c r="G35" s="14" t="n">
-        <v>178</v>
+        <v>149</v>
       </c>
       <c r="H35" s="15" t="n">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="I35" s="13">
         <f>IF($H$35="","",IF($H$35&lt;0,-$H$35/(-$H$35+100),100/($H$35+100)))</f>
@@ -11548,7 +11548,7 @@
       </c>
       <c r="N35" s="19" t="inlineStr">
         <is>
-          <t>Model 36.0% (fair +178). Your call.</t>
+          <t>Model 40.2% (fair +149). Your call.</t>
         </is>
       </c>
       <c r="O35" s="15" t="n"/>
@@ -11584,13 +11584,13 @@
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.6396999999999999</v>
+        <v>0.5984</v>
       </c>
       <c r="G36" s="14" t="n">
-        <v>-178</v>
+        <v>-149</v>
       </c>
       <c r="H36" s="15" t="n">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="I36" s="13">
         <f>IF($H$36="","",IF($H$36&lt;0,-$H$36/(-$H$36+100),100/($H$36+100)))</f>
@@ -11614,7 +11614,7 @@
       </c>
       <c r="N36" s="19" t="inlineStr">
         <is>
-          <t>Model 64.0% (fair -178). Your call.</t>
+          <t>Model 59.8% (fair -149). Your call.</t>
         </is>
       </c>
       <c r="O36" s="15" t="n"/>
@@ -11650,10 +11650,10 @@
         </is>
       </c>
       <c r="F37" s="13" t="n">
-        <v>0.3047037037037037</v>
+        <v>0.3071111111111111</v>
       </c>
       <c r="G37" s="14" t="n">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="H37" s="15" t="n">
         <v>170</v>
@@ -11680,7 +11680,7 @@
       </c>
       <c r="N37" s="19" t="inlineStr">
         <is>
-          <t>Model 30.5% (fair +228). Your call.</t>
+          <t>Model 30.7% (fair +226). Your call.</t>
         </is>
       </c>
       <c r="O37" s="15" t="n"/>
@@ -11716,13 +11716,13 @@
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.6952962962962962</v>
+        <v>0.6928897338403042</v>
       </c>
       <c r="G38" s="14" t="n">
-        <v>-228</v>
+        <v>-226</v>
       </c>
       <c r="H38" s="15" t="n">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="I38" s="13">
         <f>IF($H$38="","",IF($H$38&lt;0,-$H$38/(-$H$38+100),100/($H$38+100)))</f>
@@ -11746,7 +11746,7 @@
       </c>
       <c r="N38" s="19" t="inlineStr">
         <is>
-          <t>Model 69.5% (fair -228). Your call.</t>
+          <t>Model 69.3% (fair -226). Your call.</t>
         </is>
       </c>
       <c r="O38" s="15" t="n"/>
@@ -11782,13 +11782,13 @@
         </is>
       </c>
       <c r="F39" s="13" t="n">
-        <v>0.564118487394958</v>
+        <v>0.5629573770491804</v>
       </c>
       <c r="G39" s="14" t="n">
         <v>-129</v>
       </c>
       <c r="H39" s="15" t="n">
-        <v>-138</v>
+        <v>-144</v>
       </c>
       <c r="I39" s="13">
         <f>IF($H$39="","",IF($H$39&lt;0,-$H$39/(-$H$39+100),100/($H$39+100)))</f>
@@ -11812,7 +11812,7 @@
       </c>
       <c r="N39" s="19" t="inlineStr">
         <is>
-          <t>Model 56.4% (fair -129). Your call.</t>
+          <t>Model 56.3% (fair -129). Your call.</t>
         </is>
       </c>
       <c r="O39" s="15" t="n"/>
@@ -11848,13 +11848,13 @@
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.4358606557377049</v>
+        <v>0.4370168067226891</v>
       </c>
       <c r="G40" s="14" t="n">
         <v>129</v>
       </c>
       <c r="H40" s="15" t="n">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="I40" s="13">
         <f>IF($H$40="","",IF($H$40&lt;0,-$H$40/(-$H$40+100),100/($H$40+100)))</f>
@@ -11878,7 +11878,7 @@
       </c>
       <c r="N40" s="19" t="inlineStr">
         <is>
-          <t>Model 43.6% (fair +129). Your call.</t>
+          <t>Model 43.7% (fair +129). Your call.</t>
         </is>
       </c>
       <c r="O40" s="15" t="n"/>
@@ -12046,13 +12046,13 @@
         </is>
       </c>
       <c r="F43" s="13" t="n">
-        <v>0.5508352112676056</v>
+        <v>0.5501207547169812</v>
       </c>
       <c r="G43" s="14" t="n">
-        <v>-123</v>
+        <v>-122</v>
       </c>
       <c r="H43" s="15" t="n">
-        <v>-113</v>
+        <v>-112</v>
       </c>
       <c r="I43" s="13">
         <f>IF($H$43="","",IF($H$43&lt;0,-$H$43/(-$H$43+100),100/($H$43+100)))</f>
@@ -12076,7 +12076,7 @@
       </c>
       <c r="N43" s="19" t="inlineStr">
         <is>
-          <t>Model 55.1% (fair -123). Your call.</t>
+          <t>Model 55.0% (fair -122). Your call.</t>
         </is>
       </c>
       <c r="O43" s="15" t="n"/>
@@ -12112,10 +12112,10 @@
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>0.4491943127962085</v>
+        <v>0.4498578199052132</v>
       </c>
       <c r="G44" s="14" t="n">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H44" s="15" t="n">
         <v>111</v>
@@ -12142,7 +12142,7 @@
       </c>
       <c r="N44" s="19" t="inlineStr">
         <is>
-          <t>Model 44.9% (fair +123). Your call.</t>
+          <t>Model 45.0% (fair +122). Your call.</t>
         </is>
       </c>
       <c r="O44" s="15" t="n"/>
@@ -12178,13 +12178,13 @@
         </is>
       </c>
       <c r="F45" s="13" t="n">
-        <v>0.5065517241379309</v>
+        <v>0.50895</v>
       </c>
       <c r="G45" s="14" t="n">
-        <v>-103</v>
+        <v>-104</v>
       </c>
       <c r="H45" s="15" t="n">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="I45" s="13">
         <f>IF($H$45="","",IF($H$45&lt;0,-$H$45/(-$H$45+100),100/($H$45+100)))</f>
@@ -12208,7 +12208,7 @@
       </c>
       <c r="N45" s="19" t="inlineStr">
         <is>
-          <t>Model 50.7% (fair -103). Your call.</t>
+          <t>Model 50.9% (fair -104). Your call.</t>
         </is>
       </c>
       <c r="O45" s="15" t="n"/>
@@ -12244,10 +12244,10 @@
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.49345</v>
+        <v>0.49105</v>
       </c>
       <c r="G46" s="14" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H46" s="15" t="n">
         <v>100</v>
@@ -12274,7 +12274,7 @@
       </c>
       <c r="N46" s="19" t="inlineStr">
         <is>
-          <t>Model 49.3% (fair +103). Your call.</t>
+          <t>Model 49.1% (fair +104). Your call.</t>
         </is>
       </c>
       <c r="O46" s="15" t="n"/>
@@ -12310,10 +12310,10 @@
         </is>
       </c>
       <c r="F47" s="13" t="n">
-        <v>0.5085784313725491</v>
+        <v>0.5117156862745098</v>
       </c>
       <c r="G47" s="14" t="n">
-        <v>-103</v>
+        <v>-105</v>
       </c>
       <c r="H47" s="15" t="n">
         <v>104</v>
@@ -12340,7 +12340,7 @@
       </c>
       <c r="N47" s="19" t="inlineStr">
         <is>
-          <t>Model 50.9% (fair -103). Your call.</t>
+          <t>Model 51.2% (fair -105). Your call.</t>
         </is>
       </c>
       <c r="O47" s="15" t="n"/>
@@ -12376,13 +12376,13 @@
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>0.4914</v>
+        <v>0.4882671641791045</v>
       </c>
       <c r="G48" s="14" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H48" s="15" t="n">
-        <v>-105</v>
+        <v>-101</v>
       </c>
       <c r="I48" s="13">
         <f>IF($H$48="","",IF($H$48&lt;0,-$H$48/(-$H$48+100),100/($H$48+100)))</f>
@@ -12406,7 +12406,7 @@
       </c>
       <c r="N48" s="19" t="inlineStr">
         <is>
-          <t>Model 49.1% (fair +104). Your call.</t>
+          <t>Model 48.8% (fair +105). Your call.</t>
         </is>
       </c>
       <c r="O48" s="15" t="n"/>
@@ -12580,7 +12580,7 @@
         <v>119</v>
       </c>
       <c r="H51" s="15" t="n">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="I51" s="13">
         <f>IF($H$51="","",IF($H$51&lt;0,-$H$51/(-$H$51+100),100/($H$51+100)))</f>
@@ -12970,13 +12970,13 @@
         </is>
       </c>
       <c r="F57" s="13" t="n">
-        <v>0.4555299539170507</v>
+        <v>0.4547706422018349</v>
       </c>
       <c r="G57" s="14" t="n">
         <v>120</v>
       </c>
       <c r="H57" s="15" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="I57" s="13">
         <f>IF($H$57="","",IF($H$57&lt;0,-$H$57/(-$H$57+100),100/($H$57+100)))</f>
@@ -13000,7 +13000,7 @@
       </c>
       <c r="N57" s="19" t="inlineStr">
         <is>
-          <t>Model 45.6% (fair +120). Your call.</t>
+          <t>Model 45.5% (fair +120). Your call.</t>
         </is>
       </c>
       <c r="O57" s="15" t="n"/>
@@ -13036,7 +13036,7 @@
         </is>
       </c>
       <c r="F58" s="13" t="n">
-        <v>0.5444543778801844</v>
+        <v>0.5452092165898618</v>
       </c>
       <c r="G58" s="14" t="n">
         <v>-120</v>
@@ -13066,7 +13066,7 @@
       </c>
       <c r="N58" s="19" t="inlineStr">
         <is>
-          <t>Model 54.4% (fair -120). Your call.</t>
+          <t>Model 54.5% (fair -120). Your call.</t>
         </is>
       </c>
       <c r="O58" s="15" t="n"/>
@@ -13234,13 +13234,13 @@
         </is>
       </c>
       <c r="F61" s="13" t="n">
-        <v>0.4242578125</v>
+        <v>0.4242585551330798</v>
       </c>
       <c r="G61" s="14" t="n">
         <v>136</v>
       </c>
       <c r="H61" s="15" t="n">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="I61" s="13">
         <f>IF($H$61="","",IF($H$61&lt;0,-$H$61/(-$H$61+100),100/($H$61+100)))</f>
@@ -13366,10 +13366,10 @@
         </is>
       </c>
       <c r="F63" s="13" t="n">
-        <v>0.6677999999999999</v>
+        <v>0.6618000000000001</v>
       </c>
       <c r="G63" s="14" t="n">
-        <v>-201</v>
+        <v>-196</v>
       </c>
       <c r="H63" s="15" t="n"/>
       <c r="I63" s="13">
@@ -13394,7 +13394,7 @@
       </c>
       <c r="N63" s="19" t="inlineStr">
         <is>
-          <t>Model 66.8% (fair -201). Your call.</t>
+          <t>Model 66.2% (fair -196). Your call.</t>
         </is>
       </c>
       <c r="O63" s="15" t="n"/>
@@ -13430,10 +13430,10 @@
         </is>
       </c>
       <c r="F64" s="13" t="n">
-        <v>0.3322</v>
+        <v>0.3382</v>
       </c>
       <c r="G64" s="14" t="n">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="H64" s="15" t="n"/>
       <c r="I64" s="13">
@@ -13458,7 +13458,7 @@
       </c>
       <c r="N64" s="19" t="inlineStr">
         <is>
-          <t>Model 33.2% (fair +201). Your call.</t>
+          <t>Model 33.8% (fair +196). Your call.</t>
         </is>
       </c>
       <c r="O64" s="15" t="n"/>
@@ -13494,10 +13494,10 @@
         </is>
       </c>
       <c r="F65" s="13" t="n">
-        <v>0.3911</v>
+        <v>0.3893</v>
       </c>
       <c r="G65" s="14" t="n">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="H65" s="15" t="n"/>
       <c r="I65" s="13">
@@ -13522,7 +13522,7 @@
       </c>
       <c r="N65" s="19" t="inlineStr">
         <is>
-          <t>Model 39.1% (fair +156). Your call.</t>
+          <t>Model 38.9% (fair +157). Your call.</t>
         </is>
       </c>
       <c r="O65" s="15" t="n"/>
@@ -13558,10 +13558,10 @@
         </is>
       </c>
       <c r="F66" s="13" t="n">
-        <v>0.6089</v>
+        <v>0.6107</v>
       </c>
       <c r="G66" s="14" t="n">
-        <v>-156</v>
+        <v>-157</v>
       </c>
       <c r="H66" s="15" t="n"/>
       <c r="I66" s="13">
@@ -13586,7 +13586,7 @@
       </c>
       <c r="N66" s="19" t="inlineStr">
         <is>
-          <t>Model 60.9% (fair -156). Your call.</t>
+          <t>Model 61.1% (fair -157). Your call.</t>
         </is>
       </c>
       <c r="O66" s="15" t="n"/>
@@ -13750,13 +13750,13 @@
         </is>
       </c>
       <c r="F69" s="13" t="n">
-        <v>0.5913622119815668</v>
+        <v>0.5944477477477478</v>
       </c>
       <c r="G69" s="14" t="n">
-        <v>-145</v>
+        <v>-147</v>
       </c>
       <c r="H69" s="15" t="n">
-        <v>-117</v>
+        <v>-122</v>
       </c>
       <c r="I69" s="13">
         <f>IF($H$69="","",IF($H$69&lt;0,-$H$69/(-$H$69+100),100/($H$69+100)))</f>
@@ -13780,7 +13780,7 @@
       </c>
       <c r="N69" s="19" t="inlineStr">
         <is>
-          <t>Model 59.1% (fair -145). Your call.</t>
+          <t>Model 59.4% (fair -147). Your call.</t>
         </is>
       </c>
       <c r="O69" s="15" t="n"/>
@@ -13816,10 +13816,10 @@
         </is>
       </c>
       <c r="F70" s="13" t="n">
-        <v>0.4086486486486487</v>
+        <v>0.4055405405405406</v>
       </c>
       <c r="G70" s="14" t="n">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="H70" s="15" t="n">
         <v>122</v>
@@ -13846,7 +13846,7 @@
       </c>
       <c r="N70" s="19" t="inlineStr">
         <is>
-          <t>Model 40.9% (fair +145). Your call.</t>
+          <t>Model 40.6% (fair +147). Your call.</t>
         </is>
       </c>
       <c r="O70" s="15" t="n"/>
@@ -13882,10 +13882,10 @@
         </is>
       </c>
       <c r="F71" s="13" t="n">
-        <v>0.421015625</v>
+        <v>0.4183984374999999</v>
       </c>
       <c r="G71" s="14" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H71" s="15" t="n">
         <v>156</v>
@@ -13912,7 +13912,7 @@
       </c>
       <c r="N71" s="19" t="inlineStr">
         <is>
-          <t>Model 42.1% (fair +138). Your call.</t>
+          <t>Model 41.8% (fair +139). Your call.</t>
         </is>
       </c>
       <c r="O71" s="15" t="n"/>
@@ -13948,13 +13948,13 @@
         </is>
       </c>
       <c r="F72" s="13" t="n">
-        <v>0.579028125</v>
+        <v>0.5815939163498098</v>
       </c>
       <c r="G72" s="14" t="n">
-        <v>-138</v>
+        <v>-139</v>
       </c>
       <c r="H72" s="15" t="n">
-        <v>-156</v>
+        <v>-163</v>
       </c>
       <c r="I72" s="13">
         <f>IF($H$72="","",IF($H$72&lt;0,-$H$72/(-$H$72+100),100/($H$72+100)))</f>
@@ -13978,7 +13978,7 @@
       </c>
       <c r="N72" s="19" t="inlineStr">
         <is>
-          <t>Model 57.9% (fair -138). Your call.</t>
+          <t>Model 58.2% (fair -139). Your call.</t>
         </is>
       </c>
       <c r="O72" s="15" t="n"/>
@@ -14014,13 +14014,13 @@
         </is>
       </c>
       <c r="F73" s="13" t="n">
-        <v>0.4866346153846154</v>
+        <v>0.4828169014084507</v>
       </c>
       <c r="G73" s="14" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="H73" s="15" t="n">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="I73" s="13">
         <f>IF($H$73="","",IF($H$73&lt;0,-$H$73/(-$H$73+100),100/($H$73+100)))</f>
@@ -14044,7 +14044,7 @@
       </c>
       <c r="N73" s="19" t="inlineStr">
         <is>
-          <t>Model 48.7% (fair +105). Your call.</t>
+          <t>Model 48.3% (fair +107). Your call.</t>
         </is>
       </c>
       <c r="O73" s="15" t="n"/>
@@ -14080,10 +14080,10 @@
         </is>
       </c>
       <c r="F74" s="13" t="n">
-        <v>0.5133442396313364</v>
+        <v>0.517226267281106</v>
       </c>
       <c r="G74" s="14" t="n">
-        <v>-105</v>
+        <v>-107</v>
       </c>
       <c r="H74" s="15" t="n">
         <v>-117</v>
@@ -14110,7 +14110,7 @@
       </c>
       <c r="N74" s="19" t="inlineStr">
         <is>
-          <t>Model 51.3% (fair -105). Your call.</t>
+          <t>Model 51.7% (fair -107). Your call.</t>
         </is>
       </c>
       <c r="O74" s="15" t="n"/>
@@ -14278,10 +14278,10 @@
         </is>
       </c>
       <c r="F77" s="13" t="n">
-        <v>0.5831</v>
+        <v>0.485793991416309</v>
       </c>
       <c r="G77" s="14" t="n">
-        <v>-140</v>
+        <v>106</v>
       </c>
       <c r="H77" s="15" t="n">
         <v>133</v>
@@ -14308,7 +14308,7 @@
       </c>
       <c r="N77" s="19" t="inlineStr">
         <is>
-          <t>Model 58.3% (fair -140). Your call.</t>
+          <t>Model 48.6% (fair +106). Your call.</t>
         </is>
       </c>
       <c r="O77" s="15" t="n"/>
@@ -14344,13 +14344,13 @@
         </is>
       </c>
       <c r="F78" s="13" t="n">
-        <v>0.4169</v>
+        <v>0.5142101321585903</v>
       </c>
       <c r="G78" s="14" t="n">
-        <v>140</v>
+        <v>-106</v>
       </c>
       <c r="H78" s="15" t="n">
-        <v>-122</v>
+        <v>-127</v>
       </c>
       <c r="I78" s="13">
         <f>IF($H$78="","",IF($H$78&lt;0,-$H$78/(-$H$78+100),100/($H$78+100)))</f>
@@ -14374,7 +14374,7 @@
       </c>
       <c r="N78" s="19" t="inlineStr">
         <is>
-          <t>Model 41.7% (fair +140). Your call.</t>
+          <t>Model 51.4% (fair -106). Your call.</t>
         </is>
       </c>
       <c r="O78" s="15" t="n"/>
@@ -14410,7 +14410,7 @@
         </is>
       </c>
       <c r="F79" s="13" t="n">
-        <v>0.49285</v>
+        <v>0.49325</v>
       </c>
       <c r="G79" s="14" t="n">
         <v>103</v>
@@ -14476,13 +14476,13 @@
         </is>
       </c>
       <c r="F80" s="13" t="n">
-        <v>0.5071326923076923</v>
+        <v>0.5067450980392156</v>
       </c>
       <c r="G80" s="14" t="n">
         <v>-103</v>
       </c>
       <c r="H80" s="15" t="n">
-        <v>-108</v>
+        <v>-104</v>
       </c>
       <c r="I80" s="13">
         <f>IF($H$80="","",IF($H$80&lt;0,-$H$80/(-$H$80+100),100/($H$80+100)))</f>
@@ -14542,13 +14542,13 @@
         </is>
       </c>
       <c r="F81" s="13" t="n">
-        <v>0.4600000000000001</v>
+        <v>0.4596313364055299</v>
       </c>
       <c r="G81" s="14" t="n">
+        <v>118</v>
+      </c>
+      <c r="H81" s="15" t="n">
         <v>117</v>
-      </c>
-      <c r="H81" s="15" t="n">
-        <v>122</v>
       </c>
       <c r="I81" s="13">
         <f>IF($H$81="","",IF($H$81&lt;0,-$H$81/(-$H$81+100),100/($H$81+100)))</f>
@@ -14572,7 +14572,7 @@
       </c>
       <c r="N81" s="19" t="inlineStr">
         <is>
-          <t>Model 46.0% (fair +117). Your call.</t>
+          <t>Model 46.0% (fair +118). Your call.</t>
         </is>
       </c>
       <c r="O81" s="15" t="n"/>
@@ -14608,13 +14608,13 @@
         </is>
       </c>
       <c r="F82" s="13" t="n">
-        <v>0.5399873873873874</v>
+        <v>0.5403933920704846</v>
       </c>
       <c r="G82" s="14" t="n">
-        <v>-117</v>
+        <v>-118</v>
       </c>
       <c r="H82" s="15" t="n">
-        <v>-122</v>
+        <v>-127</v>
       </c>
       <c r="I82" s="13">
         <f>IF($H$82="","",IF($H$82&lt;0,-$H$82/(-$H$82+100),100/($H$82+100)))</f>
@@ -14638,7 +14638,7 @@
       </c>
       <c r="N82" s="19" t="inlineStr">
         <is>
-          <t>Model 54.0% (fair -117). Your call.</t>
+          <t>Model 54.0% (fair -118). Your call.</t>
         </is>
       </c>
       <c r="O82" s="15" t="n"/>
@@ -14674,10 +14674,10 @@
         </is>
       </c>
       <c r="F83" s="13" t="n">
-        <v>0.4555</v>
+        <v>0.4605</v>
       </c>
       <c r="G83" s="14" t="n">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="H83" s="15" t="n">
         <v>163</v>
@@ -14704,7 +14704,7 @@
       </c>
       <c r="N83" s="19" t="inlineStr">
         <is>
-          <t>Model 45.6% (fair +120). Your call.</t>
+          <t>Model 46.1% (fair +117). Your call.</t>
         </is>
       </c>
       <c r="O83" s="15" t="n"/>
@@ -14740,10 +14740,10 @@
         </is>
       </c>
       <c r="F84" s="13" t="n">
-        <v>0.5445</v>
+        <v>0.5395</v>
       </c>
       <c r="G84" s="14" t="n">
-        <v>-120</v>
+        <v>-117</v>
       </c>
       <c r="H84" s="15" t="n">
         <v>-127</v>
@@ -14770,7 +14770,7 @@
       </c>
       <c r="N84" s="19" t="inlineStr">
         <is>
-          <t>Model 54.4% (fair -120). Your call.</t>
+          <t>Model 53.9% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O84" s="15" t="n"/>
@@ -14806,10 +14806,10 @@
         </is>
       </c>
       <c r="F85" s="13" t="n">
-        <v>0.4079087452471483</v>
+        <v>0.4073003802281369</v>
       </c>
       <c r="G85" s="14" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H85" s="15" t="n">
         <v>163</v>
@@ -14836,7 +14836,7 @@
       </c>
       <c r="N85" s="19" t="inlineStr">
         <is>
-          <t>Model 40.8% (fair +145). Your call.</t>
+          <t>Model 40.7% (fair +146). Your call.</t>
         </is>
       </c>
       <c r="O85" s="15" t="n"/>
@@ -14872,10 +14872,10 @@
         </is>
       </c>
       <c r="F86" s="13" t="n">
-        <v>0.5920680608365019</v>
+        <v>0.5926878326996198</v>
       </c>
       <c r="G86" s="14" t="n">
-        <v>-145</v>
+        <v>-146</v>
       </c>
       <c r="H86" s="15" t="n">
         <v>-163</v>
@@ -14902,7 +14902,7 @@
       </c>
       <c r="N86" s="19" t="inlineStr">
         <is>
-          <t>Model 59.2% (fair -145). Your call.</t>
+          <t>Model 59.3% (fair -146). Your call.</t>
         </is>
       </c>
       <c r="O86" s="15" t="n"/>
@@ -14938,10 +14938,10 @@
         </is>
       </c>
       <c r="F87" s="13" t="n">
-        <v>0.5477</v>
+        <v>0.5449000000000001</v>
       </c>
       <c r="G87" s="14" t="n">
-        <v>-121</v>
+        <v>-120</v>
       </c>
       <c r="H87" s="15" t="n"/>
       <c r="I87" s="13">
@@ -14966,7 +14966,7 @@
       </c>
       <c r="N87" s="19" t="inlineStr">
         <is>
-          <t>Model 54.8% (fair -121). Your call.</t>
+          <t>Model 54.5% (fair -120). Your call.</t>
         </is>
       </c>
       <c r="O87" s="15" t="n"/>
@@ -15002,10 +15002,10 @@
         </is>
       </c>
       <c r="F88" s="13" t="n">
-        <v>0.4523</v>
+        <v>0.4551</v>
       </c>
       <c r="G88" s="14" t="n">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H88" s="15" t="n"/>
       <c r="I88" s="13">
@@ -15030,7 +15030,7 @@
       </c>
       <c r="N88" s="19" t="inlineStr">
         <is>
-          <t>Model 45.2% (fair +121). Your call.</t>
+          <t>Model 45.5% (fair +120). Your call.</t>
         </is>
       </c>
       <c r="O88" s="15" t="n"/>
@@ -15066,13 +15066,13 @@
         </is>
       </c>
       <c r="F89" s="13" t="n">
-        <v>0.5815475409836066</v>
+        <v>0.5842200000000001</v>
       </c>
       <c r="G89" s="14" t="n">
-        <v>-139</v>
+        <v>-141</v>
       </c>
       <c r="H89" s="15" t="n">
-        <v>-144</v>
+        <v>-150</v>
       </c>
       <c r="I89" s="13">
         <f>IF($H$89="","",IF($H$89&lt;0,-$H$89/(-$H$89+100),100/($H$89+100)))</f>
@@ -15096,7 +15096,7 @@
       </c>
       <c r="N89" s="19" t="inlineStr">
         <is>
-          <t>Model 58.2% (fair -139). Your call.</t>
+          <t>Model 58.4% (fair -141). Your call.</t>
         </is>
       </c>
       <c r="O89" s="15" t="n"/>
@@ -15132,10 +15132,10 @@
         </is>
       </c>
       <c r="F90" s="13" t="n">
-        <v>0.4184234234234235</v>
+        <v>0.4158108108108109</v>
       </c>
       <c r="G90" s="14" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H90" s="15" t="n">
         <v>122</v>
@@ -15162,7 +15162,7 @@
       </c>
       <c r="N90" s="19" t="inlineStr">
         <is>
-          <t>Model 41.8% (fair +139). Your call.</t>
+          <t>Model 41.6% (fair +140). Your call.</t>
         </is>
       </c>
       <c r="O90" s="15" t="n"/>
@@ -15198,13 +15198,13 @@
         </is>
       </c>
       <c r="F91" s="13" t="n">
-        <v>0.5353153153153154</v>
+        <v>0.5352995391705069</v>
       </c>
       <c r="G91" s="14" t="n">
         <v>-115</v>
       </c>
       <c r="H91" s="15" t="n">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="I91" s="13">
         <f>IF($H$91="","",IF($H$91&lt;0,-$H$91/(-$H$91+100),100/($H$91+100)))</f>
@@ -15584,7 +15584,7 @@
         </is>
       </c>
       <c r="F97" s="13" t="n">
-        <v>0.363</v>
+        <v>0.3641</v>
       </c>
       <c r="G97" s="14" t="n">
         <v>175</v>
@@ -15612,7 +15612,7 @@
       </c>
       <c r="N97" s="19" t="inlineStr">
         <is>
-          <t>Model 36.3% (fair +175). Your call.</t>
+          <t>Model 36.4% (fair +175). Your call.</t>
         </is>
       </c>
       <c r="O97" s="15" t="n"/>
@@ -15648,7 +15648,7 @@
         </is>
       </c>
       <c r="F98" s="13" t="n">
-        <v>0.637</v>
+        <v>0.6359</v>
       </c>
       <c r="G98" s="14" t="n">
         <v>-175</v>
@@ -15676,7 +15676,7 @@
       </c>
       <c r="N98" s="19" t="inlineStr">
         <is>
-          <t>Model 63.7% (fair -175). Your call.</t>
+          <t>Model 63.6% (fair -175). Your call.</t>
         </is>
       </c>
       <c r="O98" s="15" t="n"/>

</xml_diff>